<commit_message>
Add Study 002 publication tables and figures
</commit_message>
<xml_diff>
--- a/research/study_002_foundation_model_comparison/analysis/statistical_outputs/anova_results.xlsx
+++ b/research/study_002_foundation_model_comparison/analysis/statistical_outputs/anova_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\3-6-2023\muawia 03-06-2026\Agentic-AI-research\research\study_002_foundation_model_comparison\analysis\statistical_outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D2C183-E138-4C8F-94DD-D35A840610D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC74EE3-7B57-40B0-81AF-9CF5FD1573AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="1056" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -681,13 +681,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -695,7 +695,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
@@ -703,7 +703,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>33</v>
       </c>
@@ -711,7 +711,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>34</v>
       </c>
@@ -719,7 +719,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
@@ -727,7 +727,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>36</v>
       </c>
@@ -735,7 +735,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>38</v>
       </c>
@@ -743,7 +743,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>40</v>
       </c>
@@ -751,7 +751,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>42</v>
       </c>
@@ -759,7 +759,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>44</v>
       </c>
@@ -767,7 +767,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>46</v>
       </c>
@@ -775,7 +775,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>47</v>
       </c>
@@ -794,15 +794,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.77734375" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -828,7 +831,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -854,7 +857,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -880,7 +883,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -906,7 +909,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -937,15 +940,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="9.5546875" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -971,7 +974,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -997,7 +1000,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -1023,7 +1026,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -1049,7 +1052,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -1077,15 +1080,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="62.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1099,7 +1102,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1113,7 +1116,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -1138,16 +1141,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
-    <col min="3" max="4" width="37.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
+    <col min="3" max="4" width="37.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1176,7 +1179,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1205,7 +1208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1234,7 +1237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1263,7 +1266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1292,7 +1295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1321,7 +1324,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1350,7 +1353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1379,7 +1382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1408,7 +1411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1437,7 +1440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1466,7 +1469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1495,7 +1498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1524,7 +1527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -1582,7 +1585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -1611,7 +1614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -1640,7 +1643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -1669,7 +1672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -1698,7 +1701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -1727,7 +1730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -1756,7 +1759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -1785,7 +1788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>9</v>
       </c>
@@ -1814,7 +1817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -1843,7 +1846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -1872,7 +1875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -1901,7 +1904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -1930,7 +1933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -1959,7 +1962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>9</v>
       </c>
@@ -1988,7 +1991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -2017,7 +2020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -2046,7 +2049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>9</v>
       </c>
@@ -2075,7 +2078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>9</v>
       </c>
@@ -2104,7 +2107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>9</v>
       </c>
@@ -2133,7 +2136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>9</v>
       </c>
@@ -2162,7 +2165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>9</v>
       </c>
@@ -2191,7 +2194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>9</v>
       </c>
@@ -2220,7 +2223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>9</v>
       </c>
@@ -2249,7 +2252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>9</v>
       </c>
@@ -2278,7 +2281,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>9</v>
       </c>
@@ -2307,7 +2310,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>9</v>
       </c>
@@ -2336,7 +2339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>9</v>
       </c>
@@ -2365,7 +2368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>9</v>
       </c>
@@ -2394,7 +2397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -2423,7 +2426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>28</v>
       </c>
@@ -2452,7 +2455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>28</v>
       </c>
@@ -2481,7 +2484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>28</v>
       </c>
@@ -2510,7 +2513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>28</v>
       </c>
@@ -2539,7 +2542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>28</v>
       </c>
@@ -2579,16 +2582,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" customWidth="1"/>
+    <col min="2" max="2" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2608,7 +2611,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2628,7 +2631,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2648,7 +2651,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2668,7 +2671,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -2688,7 +2691,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -2708,7 +2711,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>28</v>
       </c>

</xml_diff>